<commit_message>
docs: GDD v0.3 + 아키텍처 v2.0 — 맵 커뮤니티/StatData/UIRoot/SQLite 설계 확정
</commit_message>
<xml_diff>
--- a/Assets/_Project/Data/Excel/GameData.xlsx
+++ b/Assets/_Project/Data/Excel/GameData.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="27">
   <si>
     <t>id</t>
   </si>
@@ -92,6 +92,9 @@
   </si>
   <si>
     <t>cooldown</t>
+  </si>
+  <si>
+    <t>enemy_buff_multiplier</t>
   </si>
 </sst>
 </file>
@@ -1243,7 +1246,7 @@
         <v>50.0</v>
       </c>
       <c r="I2" s="1">
-        <v>2.5</v>
+        <v>5.0</v>
       </c>
       <c r="J2" s="1">
         <v>2.0</v>
@@ -1281,7 +1284,7 @@
         <v>50.0</v>
       </c>
       <c r="I3" s="1">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="J3" s="1">
         <v>1.5</v>
@@ -1319,7 +1322,7 @@
         <v>30.0</v>
       </c>
       <c r="I4" s="1">
-        <v>3.0</v>
+        <v>6.0</v>
       </c>
       <c r="J4" s="1">
         <v>2.5</v>
@@ -1405,6 +1408,10 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="7" max="7" width="23.75"/>
+    <col customWidth="1" min="8" max="8" width="28.88"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
@@ -1428,6 +1435,9 @@
       <c r="G1" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="H1" s="1" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1">
@@ -1451,6 +1461,9 @@
       <c r="G2" s="1">
         <v>1.0</v>
       </c>
+      <c r="H2" s="1">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1">
@@ -1474,6 +1487,9 @@
       <c r="G3" s="1">
         <v>1.0</v>
       </c>
+      <c r="H3" s="1">
+        <v>1.09</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1">
@@ -1496,6 +1512,9 @@
       </c>
       <c r="G4" s="1">
         <v>1.0</v>
+      </c>
+      <c r="H4" s="1">
+        <v>1.18</v>
       </c>
     </row>
     <row r="5">
@@ -1520,6 +1539,9 @@
       <c r="G5" s="1">
         <v>1.0</v>
       </c>
+      <c r="H5" s="1">
+        <v>1.27</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1">
@@ -1543,6 +1565,9 @@
       <c r="G6" s="1">
         <v>1.0</v>
       </c>
+      <c r="H6" s="1">
+        <v>1.36</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1">
@@ -1566,6 +1591,9 @@
       <c r="G7" s="1">
         <v>1.0</v>
       </c>
+      <c r="H7" s="1">
+        <v>1.45</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1">
@@ -1589,6 +1617,9 @@
       <c r="G8" s="1">
         <v>1.0</v>
       </c>
+      <c r="H8" s="1">
+        <v>1.54</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1">
@@ -1612,6 +1643,9 @@
       <c r="G9" s="1">
         <v>1.0</v>
       </c>
+      <c r="H9" s="1">
+        <v>1.63</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1">
@@ -1635,6 +1669,9 @@
       <c r="G10" s="1">
         <v>1.0</v>
       </c>
+      <c r="H10" s="1">
+        <v>1.72</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1">
@@ -1658,6 +1695,9 @@
       <c r="G11" s="1">
         <v>1.0</v>
       </c>
+      <c r="H11" s="1">
+        <v>1.81</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1">
@@ -1681,6 +1721,9 @@
       <c r="G12" s="1">
         <v>1.0</v>
       </c>
+      <c r="H12" s="1">
+        <v>1.9</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1">
@@ -1704,6 +1747,9 @@
       <c r="G13" s="1">
         <v>1.0</v>
       </c>
+      <c r="H13" s="1">
+        <v>1.9</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1">
@@ -1727,6 +1773,9 @@
       <c r="G14" s="1">
         <v>1.0</v>
       </c>
+      <c r="H14" s="1">
+        <v>1.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1">
@@ -1750,6 +1799,9 @@
       <c r="G15" s="1">
         <v>1.0</v>
       </c>
+      <c r="H15" s="1">
+        <v>1.99</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1">
@@ -1773,6 +1825,9 @@
       <c r="G16" s="1">
         <v>1.0</v>
       </c>
+      <c r="H16" s="1">
+        <v>2.08</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1">
@@ -1796,6 +1851,9 @@
       <c r="G17" s="1">
         <v>1.0</v>
       </c>
+      <c r="H17" s="1">
+        <v>2.08</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1">
@@ -1819,6 +1877,9 @@
       <c r="G18" s="1">
         <v>1.0</v>
       </c>
+      <c r="H18" s="1">
+        <v>2.17</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1">
@@ -1842,6 +1903,9 @@
       <c r="G19" s="1">
         <v>1.0</v>
       </c>
+      <c r="H19" s="1">
+        <v>2.17</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1">
@@ -1865,6 +1929,9 @@
       <c r="G20" s="1">
         <v>1.0</v>
       </c>
+      <c r="H20" s="1">
+        <v>2.26</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1">
@@ -1888,6 +1955,9 @@
       <c r="G21" s="1">
         <v>1.0</v>
       </c>
+      <c r="H21" s="1">
+        <v>2.26</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1">
@@ -1911,6 +1981,9 @@
       <c r="G22" s="1">
         <v>1.0</v>
       </c>
+      <c r="H22" s="1">
+        <v>2.35</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="1">
@@ -1934,6 +2007,9 @@
       <c r="G23" s="1">
         <v>1.0</v>
       </c>
+      <c r="H23" s="1">
+        <v>2.35</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1">
@@ -1957,6 +2033,9 @@
       <c r="G24" s="1">
         <v>1.0</v>
       </c>
+      <c r="H24" s="1">
+        <v>2.44</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1">
@@ -1980,6 +2059,9 @@
       <c r="G25" s="1">
         <v>1.0</v>
       </c>
+      <c r="H25" s="1">
+        <v>2.44</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="1">
@@ -2003,6 +2085,9 @@
       <c r="G26" s="1">
         <v>1.0</v>
       </c>
+      <c r="H26" s="1">
+        <v>2.53</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="1">
@@ -2026,6 +2111,9 @@
       <c r="G27" s="1">
         <v>1.0</v>
       </c>
+      <c r="H27" s="1">
+        <v>2.53</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="1">
@@ -2049,6 +2137,9 @@
       <c r="G28" s="1">
         <v>1.0</v>
       </c>
+      <c r="H28" s="1">
+        <v>2.62</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="1">
@@ -2072,6 +2163,9 @@
       <c r="G29" s="1">
         <v>1.0</v>
       </c>
+      <c r="H29" s="1">
+        <v>2.62</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="1">
@@ -2095,6 +2189,9 @@
       <c r="G30" s="1">
         <v>1.0</v>
       </c>
+      <c r="H30" s="1">
+        <v>2.71</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="1">
@@ -2118,6 +2215,9 @@
       <c r="G31" s="1">
         <v>1.0</v>
       </c>
+      <c r="H31" s="1">
+        <v>2.71</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="1">
@@ -2141,6 +2241,9 @@
       <c r="G32" s="1">
         <v>1.0</v>
       </c>
+      <c r="H32" s="1">
+        <v>2.8</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="1">
@@ -2164,6 +2267,9 @@
       <c r="G33" s="1">
         <v>1.0</v>
       </c>
+      <c r="H33" s="1">
+        <v>2.8</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="1">
@@ -2187,6 +2293,9 @@
       <c r="G34" s="1">
         <v>1.0</v>
       </c>
+      <c r="H34" s="1">
+        <v>2.89</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="1">
@@ -2210,6 +2319,9 @@
       <c r="G35" s="1">
         <v>1.0</v>
       </c>
+      <c r="H35" s="1">
+        <v>2.89</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="1">
@@ -2233,6 +2345,9 @@
       <c r="G36" s="1">
         <v>1.0</v>
       </c>
+      <c r="H36" s="1">
+        <v>2.98</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="1">
@@ -2256,6 +2371,9 @@
       <c r="G37" s="1">
         <v>1.0</v>
       </c>
+      <c r="H37" s="1">
+        <v>2.98</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="1">
@@ -2279,6 +2397,9 @@
       <c r="G38" s="1">
         <v>1.0</v>
       </c>
+      <c r="H38" s="1">
+        <v>3.07</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="1">
@@ -2302,6 +2423,9 @@
       <c r="G39" s="1">
         <v>1.0</v>
       </c>
+      <c r="H39" s="1">
+        <v>3.07</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="1">
@@ -2325,6 +2449,9 @@
       <c r="G40" s="1">
         <v>1.0</v>
       </c>
+      <c r="H40" s="1">
+        <v>3.16</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="1">
@@ -2348,6 +2475,9 @@
       <c r="G41" s="1">
         <v>1.0</v>
       </c>
+      <c r="H41" s="1">
+        <v>3.16</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="1">
@@ -2371,6 +2501,9 @@
       <c r="G42" s="1">
         <v>1.0</v>
       </c>
+      <c r="H42" s="1">
+        <v>3.25</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="1">
@@ -2394,6 +2527,9 @@
       <c r="G43" s="1">
         <v>1.0</v>
       </c>
+      <c r="H43" s="1">
+        <v>3.25</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="1">
@@ -2417,6 +2553,9 @@
       <c r="G44" s="1">
         <v>1.0</v>
       </c>
+      <c r="H44" s="1">
+        <v>3.34</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="1">
@@ -2440,6 +2579,9 @@
       <c r="G45" s="1">
         <v>1.0</v>
       </c>
+      <c r="H45" s="1">
+        <v>3.34</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="1">
@@ -2463,6 +2605,9 @@
       <c r="G46" s="1">
         <v>1.0</v>
       </c>
+      <c r="H46" s="1">
+        <v>3.43</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="1">
@@ -2486,6 +2631,9 @@
       <c r="G47" s="1">
         <v>1.0</v>
       </c>
+      <c r="H47" s="1">
+        <v>3.43</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="1">
@@ -2509,6 +2657,9 @@
       <c r="G48" s="1">
         <v>1.0</v>
       </c>
+      <c r="H48" s="1">
+        <v>3.52</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="1">
@@ -2532,6 +2683,9 @@
       <c r="G49" s="1">
         <v>1.0</v>
       </c>
+      <c r="H49" s="1">
+        <v>3.52</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="1">
@@ -2555,6 +2709,9 @@
       <c r="G50" s="1">
         <v>1.0</v>
       </c>
+      <c r="H50" s="1">
+        <v>3.61</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="1">
@@ -2578,6 +2735,9 @@
       <c r="G51" s="1">
         <v>1.0</v>
       </c>
+      <c r="H51" s="1">
+        <v>3.61</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="1">
@@ -2601,6 +2761,9 @@
       <c r="G52" s="1">
         <v>1.0</v>
       </c>
+      <c r="H52" s="1">
+        <v>3.7</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="1">
@@ -2624,6 +2787,9 @@
       <c r="G53" s="1">
         <v>1.0</v>
       </c>
+      <c r="H53" s="1">
+        <v>3.7</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="1">
@@ -2647,6 +2813,9 @@
       <c r="G54" s="1">
         <v>1.0</v>
       </c>
+      <c r="H54" s="1">
+        <v>3.7</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="1">
@@ -2670,6 +2839,9 @@
       <c r="G55" s="1">
         <v>1.0</v>
       </c>
+      <c r="H55" s="1">
+        <v>3.79</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="1">
@@ -2693,6 +2865,9 @@
       <c r="G56" s="1">
         <v>1.0</v>
       </c>
+      <c r="H56" s="1">
+        <v>3.79</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="1">
@@ -2716,6 +2891,9 @@
       <c r="G57" s="1">
         <v>1.0</v>
       </c>
+      <c r="H57" s="1">
+        <v>3.79</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="1">
@@ -2739,6 +2917,9 @@
       <c r="G58" s="1">
         <v>1.0</v>
       </c>
+      <c r="H58" s="1">
+        <v>3.88</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="1">
@@ -2762,6 +2943,9 @@
       <c r="G59" s="1">
         <v>1.0</v>
       </c>
+      <c r="H59" s="1">
+        <v>3.88</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="1">
@@ -2785,6 +2969,9 @@
       <c r="G60" s="1">
         <v>1.0</v>
       </c>
+      <c r="H60" s="1">
+        <v>3.88</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="1">
@@ -2808,6 +2995,9 @@
       <c r="G61" s="1">
         <v>1.0</v>
       </c>
+      <c r="H61" s="1">
+        <v>3.97</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="1">
@@ -2831,6 +3021,9 @@
       <c r="G62" s="1">
         <v>1.0</v>
       </c>
+      <c r="H62" s="1">
+        <v>3.97</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="1">
@@ -2854,6 +3047,9 @@
       <c r="G63" s="1">
         <v>1.0</v>
       </c>
+      <c r="H63" s="1">
+        <v>3.97</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="1">
@@ -2877,6 +3073,9 @@
       <c r="G64" s="1">
         <v>1.0</v>
       </c>
+      <c r="H64" s="1">
+        <v>4.06</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="1">
@@ -2900,6 +3099,9 @@
       <c r="G65" s="1">
         <v>1.0</v>
       </c>
+      <c r="H65" s="1">
+        <v>4.06</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="1">
@@ -2923,6 +3125,9 @@
       <c r="G66" s="1">
         <v>1.0</v>
       </c>
+      <c r="H66" s="1">
+        <v>4.06</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="1">
@@ -2946,6 +3151,9 @@
       <c r="G67" s="1">
         <v>1.0</v>
       </c>
+      <c r="H67" s="1">
+        <v>4.15</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="1">
@@ -2969,6 +3177,9 @@
       <c r="G68" s="1">
         <v>1.0</v>
       </c>
+      <c r="H68" s="1">
+        <v>4.15</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="1">
@@ -2992,6 +3203,9 @@
       <c r="G69" s="1">
         <v>1.0</v>
       </c>
+      <c r="H69" s="1">
+        <v>4.15</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="1">
@@ -3015,6 +3229,9 @@
       <c r="G70" s="1">
         <v>1.0</v>
       </c>
+      <c r="H70" s="1">
+        <v>4.24</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="1">
@@ -3038,6 +3255,9 @@
       <c r="G71" s="1">
         <v>1.0</v>
       </c>
+      <c r="H71" s="1">
+        <v>4.24</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="1">
@@ -3061,6 +3281,9 @@
       <c r="G72" s="1">
         <v>1.0</v>
       </c>
+      <c r="H72" s="1">
+        <v>4.24</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="1">
@@ -3084,6 +3307,9 @@
       <c r="G73" s="1">
         <v>1.0</v>
       </c>
+      <c r="H73" s="1">
+        <v>4.33</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="1">
@@ -3107,6 +3333,9 @@
       <c r="G74" s="1">
         <v>1.0</v>
       </c>
+      <c r="H74" s="1">
+        <v>4.33</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="1">
@@ -3130,6 +3359,9 @@
       <c r="G75" s="1">
         <v>1.0</v>
       </c>
+      <c r="H75" s="1">
+        <v>4.33</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="1">
@@ -3153,6 +3385,9 @@
       <c r="G76" s="1">
         <v>1.0</v>
       </c>
+      <c r="H76" s="1">
+        <v>4.42</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="1">
@@ -3176,6 +3411,9 @@
       <c r="G77" s="1">
         <v>1.0</v>
       </c>
+      <c r="H77" s="1">
+        <v>4.42</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="1">
@@ -3199,6 +3437,9 @@
       <c r="G78" s="1">
         <v>1.0</v>
       </c>
+      <c r="H78" s="1">
+        <v>4.42</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="1">
@@ -3222,6 +3463,9 @@
       <c r="G79" s="1">
         <v>1.0</v>
       </c>
+      <c r="H79" s="1">
+        <v>4.51</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="1">
@@ -3245,6 +3489,9 @@
       <c r="G80" s="1">
         <v>1.0</v>
       </c>
+      <c r="H80" s="1">
+        <v>4.51</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="1">
@@ -3268,6 +3515,9 @@
       <c r="G81" s="1">
         <v>1.0</v>
       </c>
+      <c r="H81" s="1">
+        <v>4.51</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="1">
@@ -3291,6 +3541,9 @@
       <c r="G82" s="1">
         <v>1.0</v>
       </c>
+      <c r="H82" s="1">
+        <v>4.6</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="1">
@@ -3314,6 +3567,9 @@
       <c r="G83" s="1">
         <v>1.0</v>
       </c>
+      <c r="H83" s="1">
+        <v>4.6</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="1">
@@ -3337,6 +3593,9 @@
       <c r="G84" s="1">
         <v>1.0</v>
       </c>
+      <c r="H84" s="1">
+        <v>4.6</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="1">
@@ -3360,6 +3619,9 @@
       <c r="G85" s="1">
         <v>1.0</v>
       </c>
+      <c r="H85" s="1">
+        <v>4.69</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="1">
@@ -3383,6 +3645,9 @@
       <c r="G86" s="1">
         <v>1.0</v>
       </c>
+      <c r="H86" s="1">
+        <v>4.69</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="1">
@@ -3406,6 +3671,9 @@
       <c r="G87" s="1">
         <v>1.0</v>
       </c>
+      <c r="H87" s="1">
+        <v>4.69</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="1">
@@ -3429,6 +3697,9 @@
       <c r="G88" s="1">
         <v>1.0</v>
       </c>
+      <c r="H88" s="1">
+        <v>4.78</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="1">
@@ -3452,6 +3723,9 @@
       <c r="G89" s="1">
         <v>1.0</v>
       </c>
+      <c r="H89" s="1">
+        <v>4.78</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="1">
@@ -3475,6 +3749,9 @@
       <c r="G90" s="1">
         <v>1.0</v>
       </c>
+      <c r="H90" s="1">
+        <v>4.78</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="1">
@@ -3498,6 +3775,9 @@
       <c r="G91" s="1">
         <v>1.0</v>
       </c>
+      <c r="H91" s="1">
+        <v>4.87</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="1">
@@ -3521,6 +3801,9 @@
       <c r="G92" s="1">
         <v>1.0</v>
       </c>
+      <c r="H92" s="1">
+        <v>4.87</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="1">
@@ -3544,6 +3827,9 @@
       <c r="G93" s="1">
         <v>1.0</v>
       </c>
+      <c r="H93" s="1">
+        <v>4.87</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="1">
@@ -3567,6 +3853,9 @@
       <c r="G94" s="1">
         <v>1.0</v>
       </c>
+      <c r="H94" s="1">
+        <v>4.96</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="1">
@@ -3590,6 +3879,9 @@
       <c r="G95" s="1">
         <v>1.0</v>
       </c>
+      <c r="H95" s="1">
+        <v>4.96</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="1">
@@ -3613,6 +3905,9 @@
       <c r="G96" s="1">
         <v>1.0</v>
       </c>
+      <c r="H96" s="1">
+        <v>4.96</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="1">
@@ -3636,6 +3931,9 @@
       <c r="G97" s="1">
         <v>1.0</v>
       </c>
+      <c r="H97" s="1">
+        <v>5.05</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="1">
@@ -3659,6 +3957,9 @@
       <c r="G98" s="1">
         <v>1.0</v>
       </c>
+      <c r="H98" s="1">
+        <v>5.05</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="1">
@@ -3682,6 +3983,9 @@
       <c r="G99" s="1">
         <v>1.0</v>
       </c>
+      <c r="H99" s="1">
+        <v>5.05</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="1">
@@ -3705,6 +4009,9 @@
       <c r="G100" s="1">
         <v>1.0</v>
       </c>
+      <c r="H100" s="1">
+        <v>5.14</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="1">
@@ -3728,6 +4035,9 @@
       <c r="G101" s="1">
         <v>1.0</v>
       </c>
+      <c r="H101" s="1">
+        <v>5.14</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="1">
@@ -3751,6 +4061,9 @@
       <c r="G102" s="1">
         <v>1.0</v>
       </c>
+      <c r="H102" s="1">
+        <v>5.14</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="1">
@@ -3774,6 +4087,9 @@
       <c r="G103" s="1">
         <v>1.0</v>
       </c>
+      <c r="H103" s="1">
+        <v>5.23</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="1">
@@ -3797,6 +4113,9 @@
       <c r="G104" s="1">
         <v>1.0</v>
       </c>
+      <c r="H104" s="1">
+        <v>5.23</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="1">
@@ -3820,6 +4139,9 @@
       <c r="G105" s="1">
         <v>1.0</v>
       </c>
+      <c r="H105" s="1">
+        <v>5.23</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="1">
@@ -3843,6 +4165,9 @@
       <c r="G106" s="1">
         <v>1.0</v>
       </c>
+      <c r="H106" s="1">
+        <v>5.32</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="1">
@@ -3866,6 +4191,9 @@
       <c r="G107" s="1">
         <v>1.0</v>
       </c>
+      <c r="H107" s="1">
+        <v>5.32</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="1">
@@ -3889,6 +4217,9 @@
       <c r="G108" s="1">
         <v>1.0</v>
       </c>
+      <c r="H108" s="1">
+        <v>5.32</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="1">
@@ -3912,6 +4243,9 @@
       <c r="G109" s="1">
         <v>1.0</v>
       </c>
+      <c r="H109" s="1">
+        <v>5.41</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="1">
@@ -3935,6 +4269,9 @@
       <c r="G110" s="1">
         <v>1.0</v>
       </c>
+      <c r="H110" s="1">
+        <v>5.41</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="1">
@@ -3958,6 +4295,9 @@
       <c r="G111" s="1">
         <v>1.0</v>
       </c>
+      <c r="H111" s="1">
+        <v>5.41</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="1">
@@ -3981,6 +4321,9 @@
       <c r="G112" s="1">
         <v>1.0</v>
       </c>
+      <c r="H112" s="1">
+        <v>5.5</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="1">
@@ -4004,6 +4347,9 @@
       <c r="G113" s="1">
         <v>1.0</v>
       </c>
+      <c r="H113" s="1">
+        <v>5.5</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="1">
@@ -4027,6 +4373,9 @@
       <c r="G114" s="1">
         <v>1.0</v>
       </c>
+      <c r="H114" s="1">
+        <v>5.5</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="1">
@@ -4050,6 +4399,9 @@
       <c r="G115" s="1">
         <v>1.0</v>
       </c>
+      <c r="H115" s="1">
+        <v>5.59</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="1">
@@ -4073,6 +4425,9 @@
       <c r="G116" s="1">
         <v>1.0</v>
       </c>
+      <c r="H116" s="1">
+        <v>5.59</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="1">
@@ -4096,6 +4451,9 @@
       <c r="G117" s="1">
         <v>1.0</v>
       </c>
+      <c r="H117" s="1">
+        <v>5.59</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="1">
@@ -4119,6 +4477,9 @@
       <c r="G118" s="1">
         <v>1.0</v>
       </c>
+      <c r="H118" s="1">
+        <v>5.68</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="1">
@@ -4142,6 +4503,9 @@
       <c r="G119" s="1">
         <v>1.0</v>
       </c>
+      <c r="H119" s="1">
+        <v>5.68</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="1">
@@ -4165,6 +4529,9 @@
       <c r="G120" s="1">
         <v>1.0</v>
       </c>
+      <c r="H120" s="1">
+        <v>5.68</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="1">
@@ -4188,6 +4555,9 @@
       <c r="G121" s="1">
         <v>1.0</v>
       </c>
+      <c r="H121" s="1">
+        <v>5.77</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="1">
@@ -4211,6 +4581,9 @@
       <c r="G122" s="1">
         <v>1.0</v>
       </c>
+      <c r="H122" s="1">
+        <v>5.77</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="1">
@@ -4234,6 +4607,9 @@
       <c r="G123" s="1">
         <v>1.0</v>
       </c>
+      <c r="H123" s="1">
+        <v>5.77</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="1">
@@ -4257,6 +4633,9 @@
       <c r="G124" s="1">
         <v>1.0</v>
       </c>
+      <c r="H124" s="1">
+        <v>5.86</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="1">
@@ -4280,6 +4659,9 @@
       <c r="G125" s="1">
         <v>1.0</v>
       </c>
+      <c r="H125" s="1">
+        <v>5.86</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="1">
@@ -4303,6 +4685,9 @@
       <c r="G126" s="1">
         <v>1.0</v>
       </c>
+      <c r="H126" s="1">
+        <v>5.86</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="1">
@@ -4326,6 +4711,9 @@
       <c r="G127" s="1">
         <v>1.0</v>
       </c>
+      <c r="H127" s="1">
+        <v>5.95</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="1">
@@ -4349,6 +4737,9 @@
       <c r="G128" s="1">
         <v>1.0</v>
       </c>
+      <c r="H128" s="1">
+        <v>5.95</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="1">
@@ -4372,6 +4763,9 @@
       <c r="G129" s="1">
         <v>1.0</v>
       </c>
+      <c r="H129" s="1">
+        <v>5.95</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="1">
@@ -4395,6 +4789,9 @@
       <c r="G130" s="1">
         <v>1.0</v>
       </c>
+      <c r="H130" s="1">
+        <v>6.04</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="1">
@@ -4418,6 +4815,9 @@
       <c r="G131" s="1">
         <v>1.0</v>
       </c>
+      <c r="H131" s="1">
+        <v>6.04</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="1">
@@ -4441,6 +4841,9 @@
       <c r="G132" s="1">
         <v>1.0</v>
       </c>
+      <c r="H132" s="1">
+        <v>6.04</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="1">
@@ -4464,6 +4867,9 @@
       <c r="G133" s="1">
         <v>1.0</v>
       </c>
+      <c r="H133" s="1">
+        <v>6.13</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="1">
@@ -4487,6 +4893,9 @@
       <c r="G134" s="1">
         <v>1.0</v>
       </c>
+      <c r="H134" s="1">
+        <v>6.13</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="1">
@@ -4510,6 +4919,9 @@
       <c r="G135" s="1">
         <v>1.0</v>
       </c>
+      <c r="H135" s="1">
+        <v>6.13</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="1">
@@ -4533,6 +4945,9 @@
       <c r="G136" s="1">
         <v>1.0</v>
       </c>
+      <c r="H136" s="1">
+        <v>6.22</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="1">
@@ -4556,6 +4971,9 @@
       <c r="G137" s="1">
         <v>1.0</v>
       </c>
+      <c r="H137" s="1">
+        <v>6.22</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="1">
@@ -4579,6 +4997,9 @@
       <c r="G138" s="1">
         <v>1.0</v>
       </c>
+      <c r="H138" s="1">
+        <v>6.22</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="1">
@@ -4602,6 +5023,9 @@
       <c r="G139" s="1">
         <v>1.0</v>
       </c>
+      <c r="H139" s="1">
+        <v>6.31</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="1">
@@ -4625,6 +5049,9 @@
       <c r="G140" s="1">
         <v>1.0</v>
       </c>
+      <c r="H140" s="1">
+        <v>6.31</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="1">
@@ -4648,6 +5075,9 @@
       <c r="G141" s="1">
         <v>1.0</v>
       </c>
+      <c r="H141" s="1">
+        <v>6.31</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="1">
@@ -4671,6 +5101,9 @@
       <c r="G142" s="1">
         <v>1.0</v>
       </c>
+      <c r="H142" s="1">
+        <v>6.4</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="1">
@@ -4694,6 +5127,9 @@
       <c r="G143" s="1">
         <v>1.0</v>
       </c>
+      <c r="H143" s="1">
+        <v>6.4</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="1">
@@ -4717,6 +5153,9 @@
       <c r="G144" s="1">
         <v>1.0</v>
       </c>
+      <c r="H144" s="1">
+        <v>6.4</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="1">
@@ -4740,6 +5179,9 @@
       <c r="G145" s="1">
         <v>1.0</v>
       </c>
+      <c r="H145" s="1">
+        <v>6.49</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="1">
@@ -4763,6 +5205,9 @@
       <c r="G146" s="1">
         <v>1.0</v>
       </c>
+      <c r="H146" s="1">
+        <v>6.49</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="1">
@@ -4786,6 +5231,9 @@
       <c r="G147" s="1">
         <v>1.0</v>
       </c>
+      <c r="H147" s="1">
+        <v>6.49</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="1">
@@ -4809,6 +5257,9 @@
       <c r="G148" s="1">
         <v>1.0</v>
       </c>
+      <c r="H148" s="1">
+        <v>6.58</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="1">
@@ -4832,6 +5283,9 @@
       <c r="G149" s="1">
         <v>1.0</v>
       </c>
+      <c r="H149" s="1">
+        <v>6.58</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="1">
@@ -4855,6 +5309,9 @@
       <c r="G150" s="1">
         <v>1.0</v>
       </c>
+      <c r="H150" s="1">
+        <v>6.58</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="1">
@@ -4878,6 +5335,9 @@
       <c r="G151" s="1">
         <v>1.0</v>
       </c>
+      <c r="H151" s="1">
+        <v>6.67</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="1">
@@ -4901,6 +5361,9 @@
       <c r="G152" s="1">
         <v>1.0</v>
       </c>
+      <c r="H152" s="1">
+        <v>6.67</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="1">
@@ -4924,6 +5387,9 @@
       <c r="G153" s="1">
         <v>1.0</v>
       </c>
+      <c r="H153" s="1">
+        <v>6.67</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="1">
@@ -4947,6 +5413,9 @@
       <c r="G154" s="1">
         <v>1.0</v>
       </c>
+      <c r="H154" s="1">
+        <v>6.76</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="1">
@@ -4970,6 +5439,9 @@
       <c r="G155" s="1">
         <v>1.0</v>
       </c>
+      <c r="H155" s="1">
+        <v>6.76</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="1">
@@ -4993,6 +5465,9 @@
       <c r="G156" s="1">
         <v>1.0</v>
       </c>
+      <c r="H156" s="1">
+        <v>6.76</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="1">
@@ -5016,6 +5491,9 @@
       <c r="G157" s="1">
         <v>1.0</v>
       </c>
+      <c r="H157" s="1">
+        <v>6.85</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="1">
@@ -5039,6 +5517,9 @@
       <c r="G158" s="1">
         <v>1.0</v>
       </c>
+      <c r="H158" s="1">
+        <v>6.85</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="1">
@@ -5062,6 +5543,9 @@
       <c r="G159" s="1">
         <v>1.0</v>
       </c>
+      <c r="H159" s="1">
+        <v>6.85</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="1">
@@ -5085,6 +5569,9 @@
       <c r="G160" s="1">
         <v>1.0</v>
       </c>
+      <c r="H160" s="1">
+        <v>6.94</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="1">
@@ -5108,6 +5595,9 @@
       <c r="G161" s="1">
         <v>1.0</v>
       </c>
+      <c r="H161" s="1">
+        <v>6.94</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="1">
@@ -5131,6 +5621,9 @@
       <c r="G162" s="1">
         <v>1.0</v>
       </c>
+      <c r="H162" s="1">
+        <v>6.94</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="1">
@@ -5154,6 +5647,9 @@
       <c r="G163" s="1">
         <v>1.0</v>
       </c>
+      <c r="H163" s="1">
+        <v>7.03</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="1">
@@ -5177,6 +5673,9 @@
       <c r="G164" s="1">
         <v>1.0</v>
       </c>
+      <c r="H164" s="1">
+        <v>7.03</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="1">
@@ -5200,6 +5699,9 @@
       <c r="G165" s="1">
         <v>1.0</v>
       </c>
+      <c r="H165" s="1">
+        <v>7.03</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="1">
@@ -5223,6 +5725,9 @@
       <c r="G166" s="1">
         <v>1.0</v>
       </c>
+      <c r="H166" s="1">
+        <v>7.12</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="1">
@@ -5246,6 +5751,9 @@
       <c r="G167" s="1">
         <v>1.0</v>
       </c>
+      <c r="H167" s="1">
+        <v>7.12</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="1">
@@ -5269,6 +5777,9 @@
       <c r="G168" s="1">
         <v>1.0</v>
       </c>
+      <c r="H168" s="1">
+        <v>7.12</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="1">
@@ -5292,6 +5803,9 @@
       <c r="G169" s="1">
         <v>1.0</v>
       </c>
+      <c r="H169" s="1">
+        <v>7.21</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="1">
@@ -5315,6 +5829,9 @@
       <c r="G170" s="1">
         <v>1.0</v>
       </c>
+      <c r="H170" s="1">
+        <v>7.21</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="1">
@@ -5338,6 +5855,9 @@
       <c r="G171" s="1">
         <v>1.0</v>
       </c>
+      <c r="H171" s="1">
+        <v>7.21</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="1">
@@ -5361,6 +5881,9 @@
       <c r="G172" s="1">
         <v>1.0</v>
       </c>
+      <c r="H172" s="1">
+        <v>7.3</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="1">
@@ -5384,6 +5907,9 @@
       <c r="G173" s="1">
         <v>1.0</v>
       </c>
+      <c r="H173" s="1">
+        <v>7.3</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="1">
@@ -5407,6 +5933,9 @@
       <c r="G174" s="1">
         <v>1.0</v>
       </c>
+      <c r="H174" s="1">
+        <v>7.3</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="1">
@@ -5430,6 +5959,9 @@
       <c r="G175" s="1">
         <v>1.0</v>
       </c>
+      <c r="H175" s="1">
+        <v>7.39</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="1">
@@ -5453,6 +5985,9 @@
       <c r="G176" s="1">
         <v>1.0</v>
       </c>
+      <c r="H176" s="1">
+        <v>7.39</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="1">
@@ -5476,6 +6011,9 @@
       <c r="G177" s="1">
         <v>1.0</v>
       </c>
+      <c r="H177" s="1">
+        <v>7.39</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="1">
@@ -5499,6 +6037,9 @@
       <c r="G178" s="1">
         <v>1.0</v>
       </c>
+      <c r="H178" s="1">
+        <v>7.48</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="1">
@@ -5522,6 +6063,9 @@
       <c r="G179" s="1">
         <v>1.0</v>
       </c>
+      <c r="H179" s="1">
+        <v>7.48</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="1">
@@ -5545,6 +6089,9 @@
       <c r="G180" s="1">
         <v>1.0</v>
       </c>
+      <c r="H180" s="1">
+        <v>7.48</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="1">
@@ -5568,6 +6115,9 @@
       <c r="G181" s="1">
         <v>1.0</v>
       </c>
+      <c r="H181" s="1">
+        <v>7.57</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="1">
@@ -5591,6 +6141,9 @@
       <c r="G182" s="1">
         <v>1.0</v>
       </c>
+      <c r="H182" s="1">
+        <v>7.57</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="1">
@@ -5614,6 +6167,9 @@
       <c r="G183" s="1">
         <v>1.0</v>
       </c>
+      <c r="H183" s="1">
+        <v>7.57</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="1">
@@ -5637,6 +6193,9 @@
       <c r="G184" s="1">
         <v>1.0</v>
       </c>
+      <c r="H184" s="1">
+        <v>7.66</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="1">
@@ -5660,6 +6219,9 @@
       <c r="G185" s="1">
         <v>1.0</v>
       </c>
+      <c r="H185" s="1">
+        <v>7.66</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="1">
@@ -5683,6 +6245,9 @@
       <c r="G186" s="1">
         <v>1.0</v>
       </c>
+      <c r="H186" s="1">
+        <v>7.66</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="1">
@@ -5706,6 +6271,9 @@
       <c r="G187" s="1">
         <v>1.0</v>
       </c>
+      <c r="H187" s="1">
+        <v>7.75</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="1">
@@ -5729,6 +6297,9 @@
       <c r="G188" s="1">
         <v>1.0</v>
       </c>
+      <c r="H188" s="1">
+        <v>7.75</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="1">
@@ -5752,6 +6323,9 @@
       <c r="G189" s="1">
         <v>1.0</v>
       </c>
+      <c r="H189" s="1">
+        <v>7.75</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="1">
@@ -5775,6 +6349,9 @@
       <c r="G190" s="1">
         <v>1.0</v>
       </c>
+      <c r="H190" s="1">
+        <v>7.84</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="1">
@@ -5798,6 +6375,9 @@
       <c r="G191" s="1">
         <v>1.0</v>
       </c>
+      <c r="H191" s="1">
+        <v>7.84</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="1">
@@ -5821,6 +6401,9 @@
       <c r="G192" s="1">
         <v>1.0</v>
       </c>
+      <c r="H192" s="1">
+        <v>7.84</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="1">
@@ -5844,6 +6427,9 @@
       <c r="G193" s="1">
         <v>1.0</v>
       </c>
+      <c r="H193" s="1">
+        <v>7.93</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="1">
@@ -5867,6 +6453,9 @@
       <c r="G194" s="1">
         <v>1.0</v>
       </c>
+      <c r="H194" s="1">
+        <v>7.93</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="1">
@@ -5890,6 +6479,9 @@
       <c r="G195" s="1">
         <v>1.0</v>
       </c>
+      <c r="H195" s="1">
+        <v>7.93</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="1">
@@ -5913,6 +6505,9 @@
       <c r="G196" s="1">
         <v>1.0</v>
       </c>
+      <c r="H196" s="1">
+        <v>8.02</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="1">
@@ -5936,6 +6531,9 @@
       <c r="G197" s="1">
         <v>1.0</v>
       </c>
+      <c r="H197" s="1">
+        <v>8.02</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="1">
@@ -5959,6 +6557,9 @@
       <c r="G198" s="1">
         <v>1.0</v>
       </c>
+      <c r="H198" s="1">
+        <v>8.02</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="1">
@@ -5982,6 +6583,9 @@
       <c r="G199" s="1">
         <v>1.0</v>
       </c>
+      <c r="H199" s="1">
+        <v>8.11</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="1">
@@ -6005,6 +6609,9 @@
       <c r="G200" s="1">
         <v>1.0</v>
       </c>
+      <c r="H200" s="1">
+        <v>8.11</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="1">
@@ -6028,6 +6635,9 @@
       <c r="G201" s="1">
         <v>1.0</v>
       </c>
+      <c r="H201" s="1">
+        <v>8.11</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="1">
@@ -6051,6 +6661,9 @@
       <c r="G202" s="1">
         <v>1.0</v>
       </c>
+      <c r="H202" s="1">
+        <v>8.2</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="1">
@@ -6074,6 +6687,9 @@
       <c r="G203" s="1">
         <v>1.0</v>
       </c>
+      <c r="H203" s="1">
+        <v>8.2</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="1">
@@ -6097,6 +6713,9 @@
       <c r="G204" s="1">
         <v>1.0</v>
       </c>
+      <c r="H204" s="1">
+        <v>8.2</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="1">
@@ -6120,6 +6739,9 @@
       <c r="G205" s="1">
         <v>1.0</v>
       </c>
+      <c r="H205" s="1">
+        <v>8.29</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="1">
@@ -6143,6 +6765,9 @@
       <c r="G206" s="1">
         <v>1.0</v>
       </c>
+      <c r="H206" s="1">
+        <v>8.29</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="1">
@@ -6166,6 +6791,9 @@
       <c r="G207" s="1">
         <v>1.0</v>
       </c>
+      <c r="H207" s="1">
+        <v>8.29</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="1">
@@ -6189,6 +6817,9 @@
       <c r="G208" s="1">
         <v>1.0</v>
       </c>
+      <c r="H208" s="1">
+        <v>8.38</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="1">
@@ -6212,6 +6843,9 @@
       <c r="G209" s="1">
         <v>1.0</v>
       </c>
+      <c r="H209" s="1">
+        <v>8.38</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="1">
@@ -6235,6 +6869,9 @@
       <c r="G210" s="1">
         <v>1.0</v>
       </c>
+      <c r="H210" s="1">
+        <v>8.38</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="1">
@@ -6258,6 +6895,9 @@
       <c r="G211" s="1">
         <v>1.0</v>
       </c>
+      <c r="H211" s="1">
+        <v>8.47</v>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="1">
@@ -6281,6 +6921,9 @@
       <c r="G212" s="1">
         <v>1.0</v>
       </c>
+      <c r="H212" s="1">
+        <v>8.47</v>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="1">
@@ -6304,6 +6947,9 @@
       <c r="G213" s="1">
         <v>1.0</v>
       </c>
+      <c r="H213" s="1">
+        <v>8.47</v>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="1">
@@ -6327,6 +6973,9 @@
       <c r="G214" s="1">
         <v>1.0</v>
       </c>
+      <c r="H214" s="1">
+        <v>8.56</v>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="1">
@@ -6350,6 +6999,9 @@
       <c r="G215" s="1">
         <v>1.0</v>
       </c>
+      <c r="H215" s="1">
+        <v>8.56</v>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="1">
@@ -6373,6 +7025,9 @@
       <c r="G216" s="1">
         <v>1.0</v>
       </c>
+      <c r="H216" s="1">
+        <v>8.56</v>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="1">
@@ -6396,6 +7051,9 @@
       <c r="G217" s="1">
         <v>1.0</v>
       </c>
+      <c r="H217" s="1">
+        <v>8.65</v>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="1">
@@ -6419,6 +7077,9 @@
       <c r="G218" s="1">
         <v>1.0</v>
       </c>
+      <c r="H218" s="1">
+        <v>8.65</v>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="1">
@@ -6442,6 +7103,9 @@
       <c r="G219" s="1">
         <v>1.0</v>
       </c>
+      <c r="H219" s="1">
+        <v>8.65</v>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="1">
@@ -6465,6 +7129,9 @@
       <c r="G220" s="1">
         <v>1.0</v>
       </c>
+      <c r="H220" s="1">
+        <v>8.74</v>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="1">
@@ -6488,6 +7155,9 @@
       <c r="G221" s="1">
         <v>1.0</v>
       </c>
+      <c r="H221" s="1">
+        <v>8.74</v>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="1">
@@ -6511,6 +7181,9 @@
       <c r="G222" s="1">
         <v>1.0</v>
       </c>
+      <c r="H222" s="1">
+        <v>8.74</v>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="1">
@@ -6534,6 +7207,9 @@
       <c r="G223" s="1">
         <v>1.0</v>
       </c>
+      <c r="H223" s="1">
+        <v>8.83</v>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="1">
@@ -6557,6 +7233,9 @@
       <c r="G224" s="1">
         <v>1.0</v>
       </c>
+      <c r="H224" s="1">
+        <v>8.83</v>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="1">
@@ -6580,6 +7259,9 @@
       <c r="G225" s="1">
         <v>1.0</v>
       </c>
+      <c r="H225" s="1">
+        <v>8.83</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="1">
@@ -6603,6 +7285,9 @@
       <c r="G226" s="1">
         <v>1.0</v>
       </c>
+      <c r="H226" s="1">
+        <v>8.92</v>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="1">
@@ -6626,6 +7311,9 @@
       <c r="G227" s="1">
         <v>1.0</v>
       </c>
+      <c r="H227" s="1">
+        <v>8.92</v>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="1">
@@ -6649,6 +7337,9 @@
       <c r="G228" s="1">
         <v>1.0</v>
       </c>
+      <c r="H228" s="1">
+        <v>8.92</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="1">
@@ -6672,6 +7363,9 @@
       <c r="G229" s="1">
         <v>1.0</v>
       </c>
+      <c r="H229" s="1">
+        <v>9.01</v>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="1">
@@ -6695,6 +7389,9 @@
       <c r="G230" s="1">
         <v>1.0</v>
       </c>
+      <c r="H230" s="1">
+        <v>9.01</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="1">
@@ -6718,6 +7415,9 @@
       <c r="G231" s="1">
         <v>1.0</v>
       </c>
+      <c r="H231" s="1">
+        <v>9.01</v>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="1">
@@ -6741,6 +7441,9 @@
       <c r="G232" s="1">
         <v>1.0</v>
       </c>
+      <c r="H232" s="1">
+        <v>9.1</v>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="1">
@@ -6764,6 +7467,9 @@
       <c r="G233" s="1">
         <v>1.0</v>
       </c>
+      <c r="H233" s="1">
+        <v>9.1</v>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="1">
@@ -6787,6 +7493,9 @@
       <c r="G234" s="1">
         <v>1.0</v>
       </c>
+      <c r="H234" s="1">
+        <v>9.1</v>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="1">
@@ -6810,6 +7519,9 @@
       <c r="G235" s="1">
         <v>1.0</v>
       </c>
+      <c r="H235" s="1">
+        <v>9.19</v>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="1">
@@ -6833,6 +7545,9 @@
       <c r="G236" s="1">
         <v>1.0</v>
       </c>
+      <c r="H236" s="1">
+        <v>9.19</v>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="1">
@@ -6856,6 +7571,9 @@
       <c r="G237" s="1">
         <v>1.0</v>
       </c>
+      <c r="H237" s="1">
+        <v>9.19</v>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="1">
@@ -6879,6 +7597,9 @@
       <c r="G238" s="1">
         <v>1.0</v>
       </c>
+      <c r="H238" s="1">
+        <v>9.28</v>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="1">
@@ -6902,6 +7623,9 @@
       <c r="G239" s="1">
         <v>1.0</v>
       </c>
+      <c r="H239" s="1">
+        <v>9.28</v>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="1">
@@ -6925,6 +7649,9 @@
       <c r="G240" s="1">
         <v>1.0</v>
       </c>
+      <c r="H240" s="1">
+        <v>9.28</v>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="1">
@@ -6948,6 +7675,9 @@
       <c r="G241" s="1">
         <v>1.0</v>
       </c>
+      <c r="H241" s="1">
+        <v>9.37</v>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="1">
@@ -6971,6 +7701,9 @@
       <c r="G242" s="1">
         <v>1.0</v>
       </c>
+      <c r="H242" s="1">
+        <v>9.37</v>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="1">
@@ -6994,6 +7727,9 @@
       <c r="G243" s="1">
         <v>1.0</v>
       </c>
+      <c r="H243" s="1">
+        <v>9.37</v>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="1">
@@ -7017,6 +7753,9 @@
       <c r="G244" s="1">
         <v>1.0</v>
       </c>
+      <c r="H244" s="1">
+        <v>9.46</v>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="1">
@@ -7040,6 +7779,9 @@
       <c r="G245" s="1">
         <v>1.0</v>
       </c>
+      <c r="H245" s="1">
+        <v>9.46</v>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="1">
@@ -7063,6 +7805,9 @@
       <c r="G246" s="1">
         <v>1.0</v>
       </c>
+      <c r="H246" s="1">
+        <v>9.46</v>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="1">
@@ -7086,6 +7831,9 @@
       <c r="G247" s="1">
         <v>1.0</v>
       </c>
+      <c r="H247" s="1">
+        <v>9.55</v>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="1">
@@ -7109,6 +7857,9 @@
       <c r="G248" s="1">
         <v>1.0</v>
       </c>
+      <c r="H248" s="1">
+        <v>9.55</v>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="1">
@@ -7132,6 +7883,9 @@
       <c r="G249" s="1">
         <v>1.0</v>
       </c>
+      <c r="H249" s="1">
+        <v>9.55</v>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="1">
@@ -7155,6 +7909,9 @@
       <c r="G250" s="1">
         <v>1.0</v>
       </c>
+      <c r="H250" s="1">
+        <v>9.64</v>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="1">
@@ -7178,6 +7935,9 @@
       <c r="G251" s="1">
         <v>1.0</v>
       </c>
+      <c r="H251" s="1">
+        <v>9.64</v>
+      </c>
     </row>
     <row r="252">
       <c r="A252" s="1">
@@ -7201,6 +7961,9 @@
       <c r="G252" s="1">
         <v>1.0</v>
       </c>
+      <c r="H252" s="1">
+        <v>9.64</v>
+      </c>
     </row>
     <row r="253">
       <c r="A253" s="1">
@@ -7224,6 +7987,9 @@
       <c r="G253" s="1">
         <v>1.0</v>
       </c>
+      <c r="H253" s="1">
+        <v>9.73</v>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="1">
@@ -7247,6 +8013,9 @@
       <c r="G254" s="1">
         <v>1.0</v>
       </c>
+      <c r="H254" s="1">
+        <v>9.73</v>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="1">
@@ -7270,6 +8039,9 @@
       <c r="G255" s="1">
         <v>1.0</v>
       </c>
+      <c r="H255" s="1">
+        <v>9.73</v>
+      </c>
     </row>
     <row r="256">
       <c r="A256" s="1">
@@ -7293,6 +8065,9 @@
       <c r="G256" s="1">
         <v>1.0</v>
       </c>
+      <c r="H256" s="1">
+        <v>9.82</v>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="1">
@@ -7316,6 +8091,9 @@
       <c r="G257" s="1">
         <v>1.0</v>
       </c>
+      <c r="H257" s="1">
+        <v>9.82</v>
+      </c>
     </row>
     <row r="258">
       <c r="A258" s="1">
@@ -7339,6 +8117,9 @@
       <c r="G258" s="1">
         <v>1.0</v>
       </c>
+      <c r="H258" s="1">
+        <v>9.82</v>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="1">
@@ -7362,6 +8143,9 @@
       <c r="G259" s="1">
         <v>1.0</v>
       </c>
+      <c r="H259" s="1">
+        <v>9.91</v>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="1">
@@ -7385,6 +8169,9 @@
       <c r="G260" s="1">
         <v>1.0</v>
       </c>
+      <c r="H260" s="1">
+        <v>9.91</v>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="1">
@@ -7407,6 +8194,9 @@
       </c>
       <c r="G261" s="1">
         <v>1.0</v>
+      </c>
+      <c r="H261" s="1">
+        <v>9.91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>